<commit_message>
formcontrol and main py changes
</commit_message>
<xml_diff>
--- a/public/metadata/Final_results.xlsx
+++ b/public/metadata/Final_results.xlsx
@@ -18,12 +18,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="166" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="168" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="169" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -504,19 +505,19 @@
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
@@ -568,7 +569,7 @@
     <xf numFmtId="0" fontId="0" fillId="32" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -577,6 +578,8 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1114,20 +1117,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.8" outlineLevelRow="7"/>
-  <cols>
-    <col width="13.45" customWidth="1" min="3" max="3"/>
-    <col width="12.55" customWidth="1" min="4" max="4"/>
-    <col width="13.45" customWidth="1" min="5" max="5"/>
-    <col width="12.55" customWidth="1" min="6" max="6"/>
-    <col width="23.2666666666667" customWidth="1" min="7" max="7"/>
-    <col width="46.55" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="23.2666666666667" customWidth="1" min="10" max="10"/>
-    <col width="46.55" customWidth="1" min="11" max="11"/>
-    <col width="10.0916666666667" customWidth="1" min="12" max="12"/>
-  </cols>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1190,16 +1181,16 @@
           <t>xxx</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="7" t="n">
         <v>45839</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="7" t="n">
         <v>46022</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="7" t="n">
         <v>45658</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="7" t="n">
         <v>45838</v>
       </c>
       <c r="G2" t="inlineStr">
@@ -1217,7 +1208,7 @@
           <t>SALES_1</t>
         </is>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="J2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1230,16 +1221,16 @@
           <t>yyy</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="7" t="n">
         <v>45870</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="7" t="n">
         <v>46021</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="7" t="n">
         <v>45689</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="7" t="n">
         <v>45838</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -1257,7 +1248,7 @@
           <t>SALES_1</t>
         </is>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="J3" t="n">
         <v>0.18</v>
       </c>
     </row>
@@ -1270,16 +1261,16 @@
           <t>aaa</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="7" t="n">
         <v>45839</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="7" t="n">
         <v>46022</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="7" t="n">
         <v>45658</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="7" t="n">
         <v>45838</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -1297,7 +1288,7 @@
           <t>SALES_1</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="J4" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1310,16 +1301,16 @@
           <t>abc</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="7" t="n">
         <v>45870</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="7" t="n">
         <v>46021</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="7" t="n">
         <v>45689</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="7" t="n">
         <v>45838</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -1337,7 +1328,7 @@
           <t>SALES_1</t>
         </is>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="J5" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1350,16 +1341,16 @@
           <t>Srujan</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="7" t="n">
         <v>45839</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="7" t="n">
         <v>46022</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="7" t="n">
         <v>45658</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="7" t="n">
         <v>45838</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -1377,7 +1368,7 @@
           <t>SALES_1</t>
         </is>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="J6" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1390,16 +1381,16 @@
           <t>Ashok</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="7" t="n">
         <v>45901</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="7" t="n">
         <v>46022</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="7" t="n">
         <v>45717</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="7" t="n">
         <v>45838</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -1417,7 +1408,7 @@
           <t>SALES_1</t>
         </is>
       </c>
-      <c r="J7" s="3" t="n">
+      <c r="J7" t="n">
         <v>0.18</v>
       </c>
     </row>
@@ -1430,16 +1421,16 @@
           <t>User_1</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="7" t="n">
         <v>45839</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="7" t="n">
         <v>46022</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="7" t="n">
         <v>45658</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="7" t="n">
         <v>45838</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -1457,12 +1448,462 @@
           <t>SALES_1</t>
         </is>
       </c>
-      <c r="J8" s="3" t="n">
+      <c r="J8" t="n">
         <v>0.2</v>
       </c>
     </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>7e22f541</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>['SEGMENT_CATEGORICAL_2', 'SEGMENT_CATEGORICAL_3']</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>['SEGMENT_NUMERICAL_3', 'SEGMENT_NUMERICAL_4']</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2a42f8c4</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>['SEGMENT_CATEGORICAL_2', 'SEGMENT_CATEGORICAL_3']</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>['SEGMENT_NUMERICAL_3', 'SEGMENT_NUMERICAL_4']</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0671cf88</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>['SEGMENT_CATEGORICAL_2', 'SEGMENT_CATEGORICAL_3']</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>['SEGMENT_NUMERICAL_3', 'SEGMENT_NUMERICAL_4']</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05835027</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>['SEGMENT_CATEGORICAL_2', 'SEGMENT_CATEGORICAL_3']</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>['SEGMENT_NUMERICAL_3', 'SEGMENT_NUMERICAL_4']</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>affb8c62</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2025-03-23</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2025-04-23</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2025-03-24</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2025-04-24</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>['SEGMENT_CATEGORICAL_2', 'SEGMENT_CATEGORICAL_3']</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>['SEGMENT_NUMERICAL_3', 'SEGMENT_NUMERICAL_4']</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ed0a32f6</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2025-03-23</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2025-04-23</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2025-03-24</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2025-04-24</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>['SEGMENT_CATEGORICAL_2', 'SEGMENT_CATEGORICAL_3']</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>['SEGMENT_NUMERICAL_3', 'SEGMENT_NUMERICAL_4']</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>b50d7b9d</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2025-03-23</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2025-04-23</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025-03-24</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2025-04-24</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>['SEGMENT_CATEGORICAL_2', 'SEGMENT_CATEGORICAL_3']</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>['SEGMENT_NUMERICAL_3', 'SEGMENT_NUMERICAL_4']</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>66be9667</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2025-03-23</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2025-04-23</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2025-03-24</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2025-04-24</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>['SEGMENT_CATEGORICAL_2', 'SEGMENT_CATEGORICAL_3']</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>['SEGMENT_NUMERICAL_3', 'SEGMENT_NUMERICAL_4']</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>e3e55549</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2025-03-23</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2025-04-23</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2025-03-24</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2025-04-24</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>['SEGMENT_CATEGORICAL_2', 'SEGMENT_CATEGORICAL_3']</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>['SEGMENT_NUMERICAL_3', 'SEGMENT_NUMERICAL_4']</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>63a1947d</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2025-03-23</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2025-04-23</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2025-03-24</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2025-04-24</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>['SEGMENT_CATEGORICAL_2', 'SEGMENT_CATEGORICAL_3']</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>['SEGMENT_NUMERICAL_3', 'SEGMENT_NUMERICAL_4']</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>SALES_1</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1472,7 +1913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2034,6 +2475,329 @@
         <v>0.475587</v>
       </c>
       <c r="K14" t="inlineStr">
+        <is>
+          <t>Not Significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>User_1</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>9.485099999999999</v>
+      </c>
+      <c r="C15" t="n">
+        <v>9.299300000000001</v>
+      </c>
+      <c r="D15" t="n">
+        <v>9.7224</v>
+      </c>
+      <c r="E15" t="n">
+        <v>9.8056</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-0.1857</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.0832</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-0.269</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-323.17</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.475587</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Not Significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>User_1</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>9.485099999999999</v>
+      </c>
+      <c r="C16" t="n">
+        <v>9.299300000000001</v>
+      </c>
+      <c r="D16" t="n">
+        <v>9.7224</v>
+      </c>
+      <c r="E16" t="n">
+        <v>9.8056</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-0.1857</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.0832</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-0.269</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-323.17</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.475587</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Not Significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>affb8c62</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Not Significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ed0a32f6</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="D18" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Not Significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>b50d7b9d</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="C19" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="D19" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="E19" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Not Significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>63a1947d</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="C20" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="D20" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Not Significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>63a1947d</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="D21" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Not Significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>63a1947d</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="C22" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="D22" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Not Significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>63a1947d</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="C23" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
         <is>
           <t>Not Significant</t>
         </is>

</xml_diff>

<commit_message>
inputs group created in controlform
</commit_message>
<xml_diff>
--- a/public/metadata/Final_results.xlsx
+++ b/public/metadata/Final_results.xlsx
@@ -1913,7 +1913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2798,6 +2798,41 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
+        <is>
+          <t>Not Significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>63a1947d</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="C24" t="n">
+        <v>4.0765</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4.0143</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
         <is>
           <t>Not Significant</t>
         </is>

</xml_diff>